<commit_message>
Add The Free 50 edition — 50 questions with upsell cards
Adds the 'free50' edition with 5 categories (Fun & Chaos, Love & Attraction,
Deep Thoughts, Group Chaos, The Final Cards), each containing 10 questions
with embedded challenges and upsell cards at position 10 of each category.
Upsell cards render a locked-card UI with a premium CTA instead of a question.

https://claude.ai/code/session_017akQtnD4cWSVrCMogHuLwe
</commit_message>
<xml_diff>
--- a/AroundTheSeneya_Questions.xlsx
+++ b/AroundTheSeneya_Questions.xlsx
@@ -31,6 +31,7 @@
     <sheet name="Who Knows Me Best" sheetId="22" state="visible" r:id="rId22"/>
     <sheet name="First Impression" sheetId="23" state="visible" r:id="rId23"/>
     <sheet name="Artist Edition" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="The Free 50" sheetId="25" state="visible" r:id="rId25"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All Questions'!$A$1:$J$1</definedName>
@@ -639,7 +640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1107"/>
+  <dimension ref="A1:J1153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -47381,6 +47382,2002 @@
       </c>
       <c r="I1107" s="13" t="inlineStr"/>
       <c r="J1107" s="13" t="inlineStr"/>
+    </row>
+    <row r="1108">
+      <c r="A1108" s="2" t="inlineStr">
+        <is>
+          <t>🆓 Free (2 Editions)</t>
+        </is>
+      </c>
+      <c r="B1108" s="2" t="inlineStr">
+        <is>
+          <t>The Free 50</t>
+        </is>
+      </c>
+      <c r="C1108" s="2" t="inlineStr">
+        <is>
+          <t>خمسون سؤال</t>
+        </is>
+      </c>
+      <c r="D1108" s="2" t="inlineStr">
+        <is>
+          <t>FUN &amp; CHAOS</t>
+        </is>
+      </c>
+      <c r="E1108" s="2" t="inlineStr">
+        <is>
+          <t>الضحك والفوضى</t>
+        </is>
+      </c>
+      <c r="F1108" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1108" s="3" t="inlineStr">
+        <is>
+          <t>What's your most delusional dream life?</t>
+        </is>
+      </c>
+      <c r="H1108" s="3" t="inlineStr">
+        <is>
+          <t>شنو الحياة delulu اللي كتحلم بها؟</t>
+        </is>
+      </c>
+      <c r="I1108" s="3" t="inlineStr"/>
+      <c r="J1108" s="3" t="inlineStr"/>
+    </row>
+    <row r="1109">
+      <c r="A1109" s="2" t="inlineStr">
+        <is>
+          <t>🆓 Free (2 Editions)</t>
+        </is>
+      </c>
+      <c r="B1109" s="2" t="inlineStr">
+        <is>
+          <t>The Free 50</t>
+        </is>
+      </c>
+      <c r="C1109" s="2" t="inlineStr">
+        <is>
+          <t>خمسون سؤال</t>
+        </is>
+      </c>
+      <c r="D1109" s="2" t="inlineStr">
+        <is>
+          <t>FUN &amp; CHAOS</t>
+        </is>
+      </c>
+      <c r="E1109" s="2" t="inlineStr">
+        <is>
+          <t>الضحك والفوضى</t>
+        </is>
+      </c>
+      <c r="F1109" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1109" s="3" t="inlineStr">
+        <is>
+          <t>Who here looks innocent but probably isn't?</t>
+        </is>
+      </c>
+      <c r="H1109" s="3" t="inlineStr">
+        <is>
+          <t>شكون هنا باين innocent ولكن غالباً لا؟</t>
+        </is>
+      </c>
+      <c r="I1109" s="3" t="inlineStr"/>
+      <c r="J1109" s="3" t="inlineStr"/>
+    </row>
+    <row r="1110">
+      <c r="A1110" s="2" t="inlineStr">
+        <is>
+          <t>🆓 Free (2 Editions)</t>
+        </is>
+      </c>
+      <c r="B1110" s="2" t="inlineStr">
+        <is>
+          <t>The Free 50</t>
+        </is>
+      </c>
+      <c r="C1110" s="2" t="inlineStr">
+        <is>
+          <t>خمسون سؤال</t>
+        </is>
+      </c>
+      <c r="D1110" s="2" t="inlineStr">
+        <is>
+          <t>FUN &amp; CHAOS</t>
+        </is>
+      </c>
+      <c r="E1110" s="2" t="inlineStr">
+        <is>
+          <t>الضحك والفوضى</t>
+        </is>
+      </c>
+      <c r="F1110" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G1110" s="3" t="inlineStr">
+        <is>
+          <t>What's the weirdest thing you did because of emotions?</t>
+        </is>
+      </c>
+      <c r="H1110" s="3" t="inlineStr">
+        <is>
+          <t>شنو أغرب حاجة درتيها بسبب المشاعر؟</t>
+        </is>
+      </c>
+      <c r="I1110" s="3" t="inlineStr">
+        <is>
+          <t>Act your most dramatic emotional moment.</t>
+        </is>
+      </c>
+      <c r="J1110" s="3" t="inlineStr">
+        <is>
+          <t>مثل أكثر لحظة درامية عشتها.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1111">
+      <c r="A1111" s="2" t="inlineStr">
+        <is>
+          <t>🆓 Free (2 Editions)</t>
+        </is>
+      </c>
+      <c r="B1111" s="2" t="inlineStr">
+        <is>
+          <t>The Free 50</t>
+        </is>
+      </c>
+      <c r="C1111" s="2" t="inlineStr">
+        <is>
+          <t>خمسون سؤال</t>
+        </is>
+      </c>
+      <c r="D1111" s="2" t="inlineStr">
+        <is>
+          <t>FUN &amp; CHAOS</t>
+        </is>
+      </c>
+      <c r="E1111" s="2" t="inlineStr">
+        <is>
+          <t>الضحك والفوضى</t>
+        </is>
+      </c>
+      <c r="F1111" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="G1111" s="3" t="inlineStr">
+        <is>
+          <t>What's your biggest \</t>
+        </is>
+      </c>
+      <c r="H1111" s="3" t="inlineStr">
+        <is>
+          <t>شنو أكبر عادة كتبيّن أنك محتاج attention؟</t>
+        </is>
+      </c>
+      <c r="I1111" s="3" t="inlineStr"/>
+      <c r="J1111" s="3" t="inlineStr"/>
+    </row>
+    <row r="1112">
+      <c r="A1112" s="2" t="inlineStr">
+        <is>
+          <t>🆓 Free (2 Editions)</t>
+        </is>
+      </c>
+      <c r="B1112" s="2" t="inlineStr">
+        <is>
+          <t>The Free 50</t>
+        </is>
+      </c>
+      <c r="C1112" s="2" t="inlineStr">
+        <is>
+          <t>خمسون سؤال</t>
+        </is>
+      </c>
+      <c r="D1112" s="2" t="inlineStr">
+        <is>
+          <t>FUN &amp; CHAOS</t>
+        </is>
+      </c>
+      <c r="E1112" s="2" t="inlineStr">
+        <is>
+          <t>الضحك والفوضى</t>
+        </is>
+      </c>
+      <c r="F1112" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G1112" s="3" t="inlineStr">
+        <is>
+          <t>Who would survive a horror movie here?</t>
+        </is>
+      </c>
+      <c r="H1112" s="3" t="inlineStr">
+        <is>
+          <t>شكون يقدر ينجا ففيلم رعب هنا؟</t>
+        </is>
+      </c>
+      <c r="I1112" s="3" t="inlineStr"/>
+      <c r="J1112" s="3" t="inlineStr"/>
+    </row>
+    <row r="1113">
+      <c r="A1113" s="2" t="inlineStr">
+        <is>
+          <t>🆓 Free (2 Editions)</t>
+        </is>
+      </c>
+      <c r="B1113" s="2" t="inlineStr">
+        <is>
+          <t>The Free 50</t>
+        </is>
+      </c>
+      <c r="C1113" s="2" t="inlineStr">
+        <is>
+          <t>خمسون سؤال</t>
+        </is>
+      </c>
+      <c r="D1113" s="2" t="inlineStr">
+        <is>
+          <t>FUN &amp; CHAOS</t>
+        </is>
+      </c>
+      <c r="E1113" s="2" t="inlineStr">
+        <is>
+          <t>الضحك والفوضى</t>
+        </is>
+      </c>
+      <c r="F1113" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="G1113" s="3" t="inlineStr">
+        <is>
+          <t>What's something embarrassing you still think about at 3AM?</t>
+        </is>
+      </c>
+      <c r="H1113" s="3" t="inlineStr">
+        <is>
+          <t>شنو الحاجة المحرجة اللي باقي كتفكر فيها فالليل؟</t>
+        </is>
+      </c>
+      <c r="I1113" s="3" t="inlineStr"/>
+      <c r="J1113" s="3" t="inlineStr"/>
+    </row>
+    <row r="1114">
+      <c r="A1114" s="2" t="inlineStr">
+        <is>
+          <t>🆓 Free (2 Editions)</t>
+        </is>
+      </c>
+      <c r="B1114" s="2" t="inlineStr">
+        <is>
+          <t>The Free 50</t>
+        </is>
+      </c>
+      <c r="C1114" s="2" t="inlineStr">
+        <is>
+          <t>خمسون سؤال</t>
+        </is>
+      </c>
+      <c r="D1114" s="2" t="inlineStr">
+        <is>
+          <t>FUN &amp; CHAOS</t>
+        </is>
+      </c>
+      <c r="E1114" s="2" t="inlineStr">
+        <is>
+          <t>الضحك والفوضى</t>
+        </is>
+      </c>
+      <c r="F1114" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="G1114" s="3" t="inlineStr">
+        <is>
+          <t>What energy do you bring into a room?</t>
+        </is>
+      </c>
+      <c r="H1114" s="3" t="inlineStr">
+        <is>
+          <t>شنو الطاقة اللي كتجيب لأي بلاصة؟</t>
+        </is>
+      </c>
+      <c r="I1114" s="3" t="inlineStr">
+        <is>
+          <t>Everyone describes you in one chaotic word.</t>
+        </is>
+      </c>
+      <c r="J1114" s="3" t="inlineStr">
+        <is>
+          <t>كل واحد يوصفك بكلمة chaotic وحدة.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1115">
+      <c r="A1115" s="2" t="inlineStr">
+        <is>
+          <t>🆓 Free (2 Editions)</t>
+        </is>
+      </c>
+      <c r="B1115" s="2" t="inlineStr">
+        <is>
+          <t>The Free 50</t>
+        </is>
+      </c>
+      <c r="C1115" s="2" t="inlineStr">
+        <is>
+          <t>خمسون سؤال</t>
+        </is>
+      </c>
+      <c r="D1115" s="2" t="inlineStr">
+        <is>
+          <t>FUN &amp; CHAOS</t>
+        </is>
+      </c>
+      <c r="E1115" s="2" t="inlineStr">
+        <is>
+          <t>الضحك والفوضى</t>
+        </is>
+      </c>
+      <c r="F1115" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="G1115" s="3" t="inlineStr">
+        <is>
+          <t>What's your funniest toxic trait?</t>
+        </is>
+      </c>
+      <c r="H1115" s="3" t="inlineStr">
+        <is>
+          <t>شنو أضحك toxic trait عندك؟</t>
+        </is>
+      </c>
+      <c r="I1115" s="3" t="inlineStr"/>
+      <c r="J1115" s="3" t="inlineStr"/>
+    </row>
+    <row r="1116">
+      <c r="A1116" s="2" t="inlineStr">
+        <is>
+          <t>🆓 Free (2 Editions)</t>
+        </is>
+      </c>
+      <c r="B1116" s="2" t="inlineStr">
+        <is>
+          <t>The Free 50</t>
+        </is>
+      </c>
+      <c r="C1116" s="2" t="inlineStr">
+        <is>
+          <t>خمسون سؤال</t>
+        </is>
+      </c>
+      <c r="D1116" s="2" t="inlineStr">
+        <is>
+          <t>FUN &amp; CHAOS</t>
+        </is>
+      </c>
+      <c r="E1116" s="2" t="inlineStr">
+        <is>
+          <t>الضحك والفوضى</t>
+        </is>
+      </c>
+      <c r="F1116" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="G1116" s="3" t="inlineStr">
+        <is>
+          <t>What's your \</t>
+        </is>
+      </c>
+      <c r="H1116" s="3" t="inlineStr">
+        <is>
+          <t>شنو الأغنية اللي كتحسسك main character؟</t>
+        </is>
+      </c>
+      <c r="I1116" s="3" t="inlineStr"/>
+      <c r="J1116" s="3" t="inlineStr"/>
+    </row>
+    <row r="1117">
+      <c r="A1117" s="2" t="inlineStr">
+        <is>
+          <t>🆓 Free (2 Editions)</t>
+        </is>
+      </c>
+      <c r="B1117" s="2" t="inlineStr">
+        <is>
+          <t>The Free 50</t>
+        </is>
+      </c>
+      <c r="C1117" s="2" t="inlineStr">
+        <is>
+          <t>خمسون سؤال</t>
+        </is>
+      </c>
+      <c r="D1117" s="2" t="inlineStr">
+        <is>
+          <t>FUN &amp; CHAOS</t>
+        </is>
+      </c>
+      <c r="E1117" s="2" t="inlineStr">
+        <is>
+          <t>الضحك والفوضى</t>
+        </is>
+      </c>
+      <c r="F1117" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="G1117" s="3" t="inlineStr">
+        <is>
+          <t>What's the dumbest reason you cried for?</t>
+        </is>
+      </c>
+      <c r="H1117" s="3" t="inlineStr">
+        <is>
+          <t>شنو أغبى سبب بكيت عليه؟</t>
+        </is>
+      </c>
+      <c r="I1117" s="3" t="inlineStr"/>
+      <c r="J1117" s="3" t="inlineStr"/>
+    </row>
+    <row r="1118">
+      <c r="A1118" s="2" t="inlineStr">
+        <is>
+          <t>🆓 Free (2 Editions)</t>
+        </is>
+      </c>
+      <c r="B1118" s="2" t="inlineStr">
+        <is>
+          <t>The Free 50</t>
+        </is>
+      </c>
+      <c r="C1118" s="2" t="inlineStr">
+        <is>
+          <t>خمسون سؤال</t>
+        </is>
+      </c>
+      <c r="D1118" s="2" t="inlineStr">
+        <is>
+          <t>LOVE &amp; ATTRACTION</t>
+        </is>
+      </c>
+      <c r="E1118" s="2" t="inlineStr">
+        <is>
+          <t>الحب والجذب</t>
+        </is>
+      </c>
+      <c r="F1118" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1118" s="3" t="inlineStr">
+        <is>
+          <t>What kind of love secretly scares you?</t>
+        </is>
+      </c>
+      <c r="H1118" s="3" t="inlineStr">
+        <is>
+          <t>شنو نوع الحب اللي كيخوفك فالسر؟</t>
+        </is>
+      </c>
+      <c r="I1118" s="3" t="inlineStr"/>
+      <c r="J1118" s="3" t="inlineStr"/>
+    </row>
+    <row r="1119">
+      <c r="A1119" s="2" t="inlineStr">
+        <is>
+          <t>🆓 Free (2 Editions)</t>
+        </is>
+      </c>
+      <c r="B1119" s="2" t="inlineStr">
+        <is>
+          <t>The Free 50</t>
+        </is>
+      </c>
+      <c r="C1119" s="2" t="inlineStr">
+        <is>
+          <t>خمسون سؤال</t>
+        </is>
+      </c>
+      <c r="D1119" s="2" t="inlineStr">
+        <is>
+          <t>LOVE &amp; ATTRACTION</t>
+        </is>
+      </c>
+      <c r="E1119" s="2" t="inlineStr">
+        <is>
+          <t>الحب والجذب</t>
+        </is>
+      </c>
+      <c r="F1119" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1119" s="3" t="inlineStr">
+        <is>
+          <t>What instantly gives you butterflies?</t>
+        </is>
+      </c>
+      <c r="H1119" s="3" t="inlineStr">
+        <is>
+          <t>شنو الحاجة اللي كتجيب ليك butterflies فوراً؟</t>
+        </is>
+      </c>
+      <c r="I1119" s="3" t="inlineStr">
+        <is>
+          <t>Describe your ideal love like a movie scene.</t>
+        </is>
+      </c>
+      <c r="J1119" s="3" t="inlineStr">
+        <is>
+          <t>وصف الحب المثالي بحال مشهد فيلم.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1120">
+      <c r="A1120" s="2" t="inlineStr">
+        <is>
+          <t>🆓 Free (2 Editions)</t>
+        </is>
+      </c>
+      <c r="B1120" s="2" t="inlineStr">
+        <is>
+          <t>The Free 50</t>
+        </is>
+      </c>
+      <c r="C1120" s="2" t="inlineStr">
+        <is>
+          <t>خمسون سؤال</t>
+        </is>
+      </c>
+      <c r="D1120" s="2" t="inlineStr">
+        <is>
+          <t>LOVE &amp; ATTRACTION</t>
+        </is>
+      </c>
+      <c r="E1120" s="2" t="inlineStr">
+        <is>
+          <t>الحب والجذب</t>
+        </is>
+      </c>
+      <c r="F1120" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G1120" s="3" t="inlineStr">
+        <is>
+          <t>Would you rather be adored peacefully or loved obsessively?</t>
+        </is>
+      </c>
+      <c r="H1120" s="3" t="inlineStr">
+        <is>
+          <t>تفضل يتحبّوك بهدوء ولا بجنون؟</t>
+        </is>
+      </c>
+      <c r="I1120" s="3" t="inlineStr"/>
+      <c r="J1120" s="3" t="inlineStr"/>
+    </row>
+    <row r="1121">
+      <c r="A1121" s="2" t="inlineStr">
+        <is>
+          <t>🆓 Free (2 Editions)</t>
+        </is>
+      </c>
+      <c r="B1121" s="2" t="inlineStr">
+        <is>
+          <t>The Free 50</t>
+        </is>
+      </c>
+      <c r="C1121" s="2" t="inlineStr">
+        <is>
+          <t>خمسون سؤال</t>
+        </is>
+      </c>
+      <c r="D1121" s="2" t="inlineStr">
+        <is>
+          <t>LOVE &amp; ATTRACTION</t>
+        </is>
+      </c>
+      <c r="E1121" s="2" t="inlineStr">
+        <is>
+          <t>الحب والجذب</t>
+        </is>
+      </c>
+      <c r="F1121" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="G1121" s="3" t="inlineStr">
+        <is>
+          <t>What's your toxic romantic habit?</t>
+        </is>
+      </c>
+      <c r="H1121" s="3" t="inlineStr">
+        <is>
+          <t>شنو العادة السامة ديالك فالحب؟</t>
+        </is>
+      </c>
+      <c r="I1121" s="3" t="inlineStr"/>
+      <c r="J1121" s="3" t="inlineStr"/>
+    </row>
+    <row r="1122">
+      <c r="A1122" s="2" t="inlineStr">
+        <is>
+          <t>🆓 Free (2 Editions)</t>
+        </is>
+      </c>
+      <c r="B1122" s="2" t="inlineStr">
+        <is>
+          <t>The Free 50</t>
+        </is>
+      </c>
+      <c r="C1122" s="2" t="inlineStr">
+        <is>
+          <t>خمسون سؤال</t>
+        </is>
+      </c>
+      <c r="D1122" s="2" t="inlineStr">
+        <is>
+          <t>LOVE &amp; ATTRACTION</t>
+        </is>
+      </c>
+      <c r="E1122" s="2" t="inlineStr">
+        <is>
+          <t>الحب والجذب</t>
+        </is>
+      </c>
+      <c r="F1122" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G1122" s="3" t="inlineStr">
+        <is>
+          <t>What kind of text can ruin your mood instantly?</t>
+        </is>
+      </c>
+      <c r="H1122" s="3" t="inlineStr">
+        <is>
+          <t>شنو نوع المساج اللي يقدر يخسر ليك المود فوراً؟</t>
+        </is>
+      </c>
+      <c r="I1122" s="3" t="inlineStr"/>
+      <c r="J1122" s="3" t="inlineStr"/>
+    </row>
+    <row r="1123">
+      <c r="A1123" s="2" t="inlineStr">
+        <is>
+          <t>🆓 Free (2 Editions)</t>
+        </is>
+      </c>
+      <c r="B1123" s="2" t="inlineStr">
+        <is>
+          <t>The Free 50</t>
+        </is>
+      </c>
+      <c r="C1123" s="2" t="inlineStr">
+        <is>
+          <t>خمسون سؤال</t>
+        </is>
+      </c>
+      <c r="D1123" s="2" t="inlineStr">
+        <is>
+          <t>LOVE &amp; ATTRACTION</t>
+        </is>
+      </c>
+      <c r="E1123" s="2" t="inlineStr">
+        <is>
+          <t>الحب والجذب</t>
+        </is>
+      </c>
+      <c r="F1123" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="G1123" s="3" t="inlineStr">
+        <is>
+          <t>What's something romantic you pretend not to want?</t>
+        </is>
+      </c>
+      <c r="H1123" s="3" t="inlineStr">
+        <is>
+          <t>شنو الحاجة الرومانسية اللي كتدير راسك ما باغيهاش؟</t>
+        </is>
+      </c>
+      <c r="I1123" s="3" t="inlineStr"/>
+      <c r="J1123" s="3" t="inlineStr"/>
+    </row>
+    <row r="1124">
+      <c r="A1124" s="2" t="inlineStr">
+        <is>
+          <t>🆓 Free (2 Editions)</t>
+        </is>
+      </c>
+      <c r="B1124" s="2" t="inlineStr">
+        <is>
+          <t>The Free 50</t>
+        </is>
+      </c>
+      <c r="C1124" s="2" t="inlineStr">
+        <is>
+          <t>خمسون سؤال</t>
+        </is>
+      </c>
+      <c r="D1124" s="2" t="inlineStr">
+        <is>
+          <t>LOVE &amp; ATTRACTION</t>
+        </is>
+      </c>
+      <c r="E1124" s="2" t="inlineStr">
+        <is>
+          <t>الحب والجذب</t>
+        </is>
+      </c>
+      <c r="F1124" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="G1124" s="3" t="inlineStr">
+        <is>
+          <t>What's your biggest fear in relationships?</t>
+        </is>
+      </c>
+      <c r="H1124" s="3" t="inlineStr">
+        <is>
+          <t>شنو أكبر خوف عندك فالعلاقات؟</t>
+        </is>
+      </c>
+      <c r="I1124" s="3" t="inlineStr"/>
+      <c r="J1124" s="3" t="inlineStr"/>
+    </row>
+    <row r="1125">
+      <c r="A1125" s="2" t="inlineStr">
+        <is>
+          <t>🆓 Free (2 Editions)</t>
+        </is>
+      </c>
+      <c r="B1125" s="2" t="inlineStr">
+        <is>
+          <t>The Free 50</t>
+        </is>
+      </c>
+      <c r="C1125" s="2" t="inlineStr">
+        <is>
+          <t>خمسون سؤال</t>
+        </is>
+      </c>
+      <c r="D1125" s="2" t="inlineStr">
+        <is>
+          <t>LOVE &amp; ATTRACTION</t>
+        </is>
+      </c>
+      <c r="E1125" s="2" t="inlineStr">
+        <is>
+          <t>الحب والجذب</t>
+        </is>
+      </c>
+      <c r="F1125" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="G1125" s="3" t="inlineStr">
+        <is>
+          <t>What makes someone emotionally attractive to you?</t>
+        </is>
+      </c>
+      <c r="H1125" s="3" t="inlineStr">
+        <is>
+          <t>شنو كيخلي الشخص جذاب نفسياً؟</t>
+        </is>
+      </c>
+      <c r="I1125" s="3" t="inlineStr"/>
+      <c r="J1125" s="3" t="inlineStr"/>
+    </row>
+    <row r="1126">
+      <c r="A1126" s="2" t="inlineStr">
+        <is>
+          <t>🆓 Free (2 Editions)</t>
+        </is>
+      </c>
+      <c r="B1126" s="2" t="inlineStr">
+        <is>
+          <t>The Free 50</t>
+        </is>
+      </c>
+      <c r="C1126" s="2" t="inlineStr">
+        <is>
+          <t>خمسون سؤال</t>
+        </is>
+      </c>
+      <c r="D1126" s="2" t="inlineStr">
+        <is>
+          <t>LOVE &amp; ATTRACTION</t>
+        </is>
+      </c>
+      <c r="E1126" s="2" t="inlineStr">
+        <is>
+          <t>الحب والجذب</t>
+        </is>
+      </c>
+      <c r="F1126" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="G1126" s="3" t="inlineStr">
+        <is>
+          <t>What kind of love story fits your soul?</t>
+        </is>
+      </c>
+      <c r="H1126" s="3" t="inlineStr">
+        <is>
+          <t>شنو قصة الحب اللي كتشبه روحك؟</t>
+        </is>
+      </c>
+      <c r="I1126" s="3" t="inlineStr"/>
+      <c r="J1126" s="3" t="inlineStr"/>
+    </row>
+    <row r="1127">
+      <c r="A1127" s="2" t="inlineStr">
+        <is>
+          <t>🆓 Free (2 Editions)</t>
+        </is>
+      </c>
+      <c r="B1127" s="2" t="inlineStr">
+        <is>
+          <t>The Free 50</t>
+        </is>
+      </c>
+      <c r="C1127" s="2" t="inlineStr">
+        <is>
+          <t>خمسون سؤال</t>
+        </is>
+      </c>
+      <c r="D1127" s="2" t="inlineStr">
+        <is>
+          <t>DEEP THOUGHTS</t>
+        </is>
+      </c>
+      <c r="E1127" s="2" t="inlineStr">
+        <is>
+          <t>أعماق التفكير</t>
+        </is>
+      </c>
+      <c r="F1127" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1127" s="3" t="inlineStr">
+        <is>
+          <t>What thought ruins your peace the most?</t>
+        </is>
+      </c>
+      <c r="H1127" s="3" t="inlineStr">
+        <is>
+          <t>شنو الفكرة اللي كتخرب عليك الراحة أكثر؟</t>
+        </is>
+      </c>
+      <c r="I1127" s="3" t="inlineStr"/>
+      <c r="J1127" s="3" t="inlineStr"/>
+    </row>
+    <row r="1128">
+      <c r="A1128" s="2" t="inlineStr">
+        <is>
+          <t>🆓 Free (2 Editions)</t>
+        </is>
+      </c>
+      <c r="B1128" s="2" t="inlineStr">
+        <is>
+          <t>The Free 50</t>
+        </is>
+      </c>
+      <c r="C1128" s="2" t="inlineStr">
+        <is>
+          <t>خمسون سؤال</t>
+        </is>
+      </c>
+      <c r="D1128" s="2" t="inlineStr">
+        <is>
+          <t>DEEP THOUGHTS</t>
+        </is>
+      </c>
+      <c r="E1128" s="2" t="inlineStr">
+        <is>
+          <t>أعماق التفكير</t>
+        </is>
+      </c>
+      <c r="F1128" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1128" s="3" t="inlineStr">
+        <is>
+          <t>What do you hide behind your personality?</t>
+        </is>
+      </c>
+      <c r="H1128" s="3" t="inlineStr">
+        <is>
+          <t>شنو كتخبي ورا شخصيتك؟</t>
+        </is>
+      </c>
+      <c r="I1128" s="3" t="inlineStr"/>
+      <c r="J1128" s="3" t="inlineStr"/>
+    </row>
+    <row r="1129">
+      <c r="A1129" s="2" t="inlineStr">
+        <is>
+          <t>🆓 Free (2 Editions)</t>
+        </is>
+      </c>
+      <c r="B1129" s="2" t="inlineStr">
+        <is>
+          <t>The Free 50</t>
+        </is>
+      </c>
+      <c r="C1129" s="2" t="inlineStr">
+        <is>
+          <t>خمسون سؤال</t>
+        </is>
+      </c>
+      <c r="D1129" s="2" t="inlineStr">
+        <is>
+          <t>DEEP THOUGHTS</t>
+        </is>
+      </c>
+      <c r="E1129" s="2" t="inlineStr">
+        <is>
+          <t>أعماق التفكير</t>
+        </is>
+      </c>
+      <c r="F1129" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G1129" s="3" t="inlineStr">
+        <is>
+          <t>What version of yourself are you grieving?</t>
+        </is>
+      </c>
+      <c r="H1129" s="3" t="inlineStr">
+        <is>
+          <t>شنو النسخة منك اللي كتحزن عليها؟</t>
+        </is>
+      </c>
+      <c r="I1129" s="3" t="inlineStr"/>
+      <c r="J1129" s="3" t="inlineStr"/>
+    </row>
+    <row r="1130">
+      <c r="A1130" s="2" t="inlineStr">
+        <is>
+          <t>🆓 Free (2 Editions)</t>
+        </is>
+      </c>
+      <c r="B1130" s="2" t="inlineStr">
+        <is>
+          <t>The Free 50</t>
+        </is>
+      </c>
+      <c r="C1130" s="2" t="inlineStr">
+        <is>
+          <t>خمسون سؤال</t>
+        </is>
+      </c>
+      <c r="D1130" s="2" t="inlineStr">
+        <is>
+          <t>DEEP THOUGHTS</t>
+        </is>
+      </c>
+      <c r="E1130" s="2" t="inlineStr">
+        <is>
+          <t>أعماق التفكير</t>
+        </is>
+      </c>
+      <c r="F1130" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="G1130" s="3" t="inlineStr">
+        <is>
+          <t>What emotional wound still affects you quietly?</t>
+        </is>
+      </c>
+      <c r="H1130" s="3" t="inlineStr">
+        <is>
+          <t>شنو الجرح اللي باقي كيأثر عليك بصمت؟</t>
+        </is>
+      </c>
+      <c r="I1130" s="3" t="inlineStr"/>
+      <c r="J1130" s="3" t="inlineStr"/>
+    </row>
+    <row r="1131">
+      <c r="A1131" s="2" t="inlineStr">
+        <is>
+          <t>🆓 Free (2 Editions)</t>
+        </is>
+      </c>
+      <c r="B1131" s="2" t="inlineStr">
+        <is>
+          <t>The Free 50</t>
+        </is>
+      </c>
+      <c r="C1131" s="2" t="inlineStr">
+        <is>
+          <t>خمسون سؤال</t>
+        </is>
+      </c>
+      <c r="D1131" s="2" t="inlineStr">
+        <is>
+          <t>DEEP THOUGHTS</t>
+        </is>
+      </c>
+      <c r="E1131" s="2" t="inlineStr">
+        <is>
+          <t>أعماق التفكير</t>
+        </is>
+      </c>
+      <c r="F1131" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G1131" s="3" t="inlineStr">
+        <is>
+          <t>What do you wish people understood about you?</t>
+        </is>
+      </c>
+      <c r="H1131" s="3" t="inlineStr">
+        <is>
+          <t>شنو بغيتي الناس يفهموه عليك؟</t>
+        </is>
+      </c>
+      <c r="I1131" s="3" t="inlineStr"/>
+      <c r="J1131" s="3" t="inlineStr"/>
+    </row>
+    <row r="1132">
+      <c r="A1132" s="2" t="inlineStr">
+        <is>
+          <t>🆓 Free (2 Editions)</t>
+        </is>
+      </c>
+      <c r="B1132" s="2" t="inlineStr">
+        <is>
+          <t>The Free 50</t>
+        </is>
+      </c>
+      <c r="C1132" s="2" t="inlineStr">
+        <is>
+          <t>خمسون سؤال</t>
+        </is>
+      </c>
+      <c r="D1132" s="2" t="inlineStr">
+        <is>
+          <t>DEEP THOUGHTS</t>
+        </is>
+      </c>
+      <c r="E1132" s="2" t="inlineStr">
+        <is>
+          <t>أعماق التفكير</t>
+        </is>
+      </c>
+      <c r="F1132" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="G1132" s="3" t="inlineStr">
+        <is>
+          <t>What's a fear you never say out loud?</t>
+        </is>
+      </c>
+      <c r="H1132" s="3" t="inlineStr">
+        <is>
+          <t>شنو الخوف اللي ما كتقولوش بصوت عالي؟</t>
+        </is>
+      </c>
+      <c r="I1132" s="3" t="inlineStr">
+        <is>
+          <t>Silence round — answer with no jokes allowed.</t>
+        </is>
+      </c>
+      <c r="J1132" s="3" t="inlineStr">
+        <is>
+          <t>جولة الصمت — جاوب بلا ضحك ولا هزار.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1133">
+      <c r="A1133" s="2" t="inlineStr">
+        <is>
+          <t>🆓 Free (2 Editions)</t>
+        </is>
+      </c>
+      <c r="B1133" s="2" t="inlineStr">
+        <is>
+          <t>The Free 50</t>
+        </is>
+      </c>
+      <c r="C1133" s="2" t="inlineStr">
+        <is>
+          <t>خمسون سؤال</t>
+        </is>
+      </c>
+      <c r="D1133" s="2" t="inlineStr">
+        <is>
+          <t>DEEP THOUGHTS</t>
+        </is>
+      </c>
+      <c r="E1133" s="2" t="inlineStr">
+        <is>
+          <t>أعماق التفكير</t>
+        </is>
+      </c>
+      <c r="F1133" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="G1133" s="3" t="inlineStr">
+        <is>
+          <t>What kind of loneliness do you experience?</t>
+        </is>
+      </c>
+      <c r="H1133" s="3" t="inlineStr">
+        <is>
+          <t>شنو نوع الوحدة اللي كتحس بها؟</t>
+        </is>
+      </c>
+      <c r="I1133" s="3" t="inlineStr"/>
+      <c r="J1133" s="3" t="inlineStr"/>
+    </row>
+    <row r="1134">
+      <c r="A1134" s="2" t="inlineStr">
+        <is>
+          <t>🆓 Free (2 Editions)</t>
+        </is>
+      </c>
+      <c r="B1134" s="2" t="inlineStr">
+        <is>
+          <t>The Free 50</t>
+        </is>
+      </c>
+      <c r="C1134" s="2" t="inlineStr">
+        <is>
+          <t>خمسون سؤال</t>
+        </is>
+      </c>
+      <c r="D1134" s="2" t="inlineStr">
+        <is>
+          <t>DEEP THOUGHTS</t>
+        </is>
+      </c>
+      <c r="E1134" s="2" t="inlineStr">
+        <is>
+          <t>أعماق التفكير</t>
+        </is>
+      </c>
+      <c r="F1134" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="G1134" s="3" t="inlineStr">
+        <is>
+          <t>What emotion do you struggle to express?</t>
+        </is>
+      </c>
+      <c r="H1134" s="3" t="inlineStr">
+        <is>
+          <t>شنو الإحساس اللي صعيب عليك تعبر عليه؟</t>
+        </is>
+      </c>
+      <c r="I1134" s="3" t="inlineStr"/>
+      <c r="J1134" s="3" t="inlineStr"/>
+    </row>
+    <row r="1135">
+      <c r="A1135" s="2" t="inlineStr">
+        <is>
+          <t>🆓 Free (2 Editions)</t>
+        </is>
+      </c>
+      <c r="B1135" s="2" t="inlineStr">
+        <is>
+          <t>The Free 50</t>
+        </is>
+      </c>
+      <c r="C1135" s="2" t="inlineStr">
+        <is>
+          <t>خمسون سؤال</t>
+        </is>
+      </c>
+      <c r="D1135" s="2" t="inlineStr">
+        <is>
+          <t>DEEP THOUGHTS</t>
+        </is>
+      </c>
+      <c r="E1135" s="2" t="inlineStr">
+        <is>
+          <t>أعماق التفكير</t>
+        </is>
+      </c>
+      <c r="F1135" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="G1135" s="3" t="inlineStr">
+        <is>
+          <t>What do you overthink the most at night?</t>
+        </is>
+      </c>
+      <c r="H1135" s="3" t="inlineStr">
+        <is>
+          <t>شنو كتكتر التفكير فيه فالليل؟</t>
+        </is>
+      </c>
+      <c r="I1135" s="3" t="inlineStr"/>
+      <c r="J1135" s="3" t="inlineStr"/>
+    </row>
+    <row r="1136">
+      <c r="A1136" s="2" t="inlineStr">
+        <is>
+          <t>🆓 Free (2 Editions)</t>
+        </is>
+      </c>
+      <c r="B1136" s="2" t="inlineStr">
+        <is>
+          <t>The Free 50</t>
+        </is>
+      </c>
+      <c r="C1136" s="2" t="inlineStr">
+        <is>
+          <t>خمسون سؤال</t>
+        </is>
+      </c>
+      <c r="D1136" s="2" t="inlineStr">
+        <is>
+          <t>GROUP CHAOS</t>
+        </is>
+      </c>
+      <c r="E1136" s="2" t="inlineStr">
+        <is>
+          <t>فوضى المجموعة</t>
+        </is>
+      </c>
+      <c r="F1136" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1136" s="3" t="inlineStr">
+        <is>
+          <t>Who here hides their emotions the best?</t>
+        </is>
+      </c>
+      <c r="H1136" s="3" t="inlineStr">
+        <is>
+          <t>شكون هنا كايخبي مشاعرو مزيان؟</t>
+        </is>
+      </c>
+      <c r="I1136" s="3" t="inlineStr"/>
+      <c r="J1136" s="3" t="inlineStr"/>
+    </row>
+    <row r="1137">
+      <c r="A1137" s="2" t="inlineStr">
+        <is>
+          <t>🆓 Free (2 Editions)</t>
+        </is>
+      </c>
+      <c r="B1137" s="2" t="inlineStr">
+        <is>
+          <t>The Free 50</t>
+        </is>
+      </c>
+      <c r="C1137" s="2" t="inlineStr">
+        <is>
+          <t>خمسون سؤال</t>
+        </is>
+      </c>
+      <c r="D1137" s="2" t="inlineStr">
+        <is>
+          <t>GROUP CHAOS</t>
+        </is>
+      </c>
+      <c r="E1137" s="2" t="inlineStr">
+        <is>
+          <t>فوضى المجموعة</t>
+        </is>
+      </c>
+      <c r="F1137" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1137" s="3" t="inlineStr">
+        <is>
+          <t>Who would fall in love the fastest?</t>
+        </is>
+      </c>
+      <c r="H1137" s="3" t="inlineStr">
+        <is>
+          <t>شكون يقدر يحب بسرعة أكثر؟</t>
+        </is>
+      </c>
+      <c r="I1137" s="3" t="inlineStr">
+        <is>
+          <t>Vote anonymously.</t>
+        </is>
+      </c>
+      <c r="J1137" s="3" t="inlineStr">
+        <is>
+          <t>صوتو anonymously.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1138">
+      <c r="A1138" s="2" t="inlineStr">
+        <is>
+          <t>🆓 Free (2 Editions)</t>
+        </is>
+      </c>
+      <c r="B1138" s="2" t="inlineStr">
+        <is>
+          <t>The Free 50</t>
+        </is>
+      </c>
+      <c r="C1138" s="2" t="inlineStr">
+        <is>
+          <t>خمسون سؤال</t>
+        </is>
+      </c>
+      <c r="D1138" s="2" t="inlineStr">
+        <is>
+          <t>GROUP CHAOS</t>
+        </is>
+      </c>
+      <c r="E1138" s="2" t="inlineStr">
+        <is>
+          <t>فوضى المجموعة</t>
+        </is>
+      </c>
+      <c r="F1138" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G1138" s="3" t="inlineStr">
+        <is>
+          <t>Who looks soft but is emotionally dangerous?</t>
+        </is>
+      </c>
+      <c r="H1138" s="3" t="inlineStr">
+        <is>
+          <t>شكون باين حنين ولكن dangerous عاطفياً؟</t>
+        </is>
+      </c>
+      <c r="I1138" s="3" t="inlineStr"/>
+      <c r="J1138" s="3" t="inlineStr"/>
+    </row>
+    <row r="1139">
+      <c r="A1139" s="2" t="inlineStr">
+        <is>
+          <t>🆓 Free (2 Editions)</t>
+        </is>
+      </c>
+      <c r="B1139" s="2" t="inlineStr">
+        <is>
+          <t>The Free 50</t>
+        </is>
+      </c>
+      <c r="C1139" s="2" t="inlineStr">
+        <is>
+          <t>خمسون سؤال</t>
+        </is>
+      </c>
+      <c r="D1139" s="2" t="inlineStr">
+        <is>
+          <t>GROUP CHAOS</t>
+        </is>
+      </c>
+      <c r="E1139" s="2" t="inlineStr">
+        <is>
+          <t>فوضى المجموعة</t>
+        </is>
+      </c>
+      <c r="F1139" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="G1139" s="3" t="inlineStr">
+        <is>
+          <t>Who gives heartbreak energy?</t>
+        </is>
+      </c>
+      <c r="H1139" s="3" t="inlineStr">
+        <is>
+          <t>شكون كييعطي heartbreak energy؟</t>
+        </is>
+      </c>
+      <c r="I1139" s="3" t="inlineStr"/>
+      <c r="J1139" s="3" t="inlineStr"/>
+    </row>
+    <row r="1140">
+      <c r="A1140" s="2" t="inlineStr">
+        <is>
+          <t>🆓 Free (2 Editions)</t>
+        </is>
+      </c>
+      <c r="B1140" s="2" t="inlineStr">
+        <is>
+          <t>The Free 50</t>
+        </is>
+      </c>
+      <c r="C1140" s="2" t="inlineStr">
+        <is>
+          <t>خمسون سؤال</t>
+        </is>
+      </c>
+      <c r="D1140" s="2" t="inlineStr">
+        <is>
+          <t>GROUP CHAOS</t>
+        </is>
+      </c>
+      <c r="E1140" s="2" t="inlineStr">
+        <is>
+          <t>فوضى المجموعة</t>
+        </is>
+      </c>
+      <c r="F1140" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G1140" s="3" t="inlineStr">
+        <is>
+          <t>Who overthinks every text message?</t>
+        </is>
+      </c>
+      <c r="H1140" s="3" t="inlineStr">
+        <is>
+          <t>شكون كيحلل كل مساج بزاف؟</t>
+        </is>
+      </c>
+      <c r="I1140" s="3" t="inlineStr"/>
+      <c r="J1140" s="3" t="inlineStr"/>
+    </row>
+    <row r="1141">
+      <c r="A1141" s="2" t="inlineStr">
+        <is>
+          <t>🆓 Free (2 Editions)</t>
+        </is>
+      </c>
+      <c r="B1141" s="2" t="inlineStr">
+        <is>
+          <t>The Free 50</t>
+        </is>
+      </c>
+      <c r="C1141" s="2" t="inlineStr">
+        <is>
+          <t>خمسون سؤال</t>
+        </is>
+      </c>
+      <c r="D1141" s="2" t="inlineStr">
+        <is>
+          <t>GROUP CHAOS</t>
+        </is>
+      </c>
+      <c r="E1141" s="2" t="inlineStr">
+        <is>
+          <t>فوضى المجموعة</t>
+        </is>
+      </c>
+      <c r="F1141" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="G1141" s="3" t="inlineStr">
+        <is>
+          <t>Who would disappear after heartbreak?</t>
+        </is>
+      </c>
+      <c r="H1141" s="3" t="inlineStr">
+        <is>
+          <t>شكون يقدر يختفي من بعد heartbreak؟</t>
+        </is>
+      </c>
+      <c r="I1141" s="3" t="inlineStr">
+        <is>
+          <t>Everyone imitates the person they choose.</t>
+        </is>
+      </c>
+      <c r="J1141" s="3" t="inlineStr">
+        <is>
+          <t>كل واحد يقلد الشخص اللي اختار.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1142">
+      <c r="A1142" s="2" t="inlineStr">
+        <is>
+          <t>🆓 Free (2 Editions)</t>
+        </is>
+      </c>
+      <c r="B1142" s="2" t="inlineStr">
+        <is>
+          <t>The Free 50</t>
+        </is>
+      </c>
+      <c r="C1142" s="2" t="inlineStr">
+        <is>
+          <t>خمسون سؤال</t>
+        </is>
+      </c>
+      <c r="D1142" s="2" t="inlineStr">
+        <is>
+          <t>GROUP CHAOS</t>
+        </is>
+      </c>
+      <c r="E1142" s="2" t="inlineStr">
+        <is>
+          <t>فوضى المجموعة</t>
+        </is>
+      </c>
+      <c r="F1142" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="G1142" s="3" t="inlineStr">
+        <is>
+          <t>Who acts emotionally unavailable but actually cares deeply?</t>
+        </is>
+      </c>
+      <c r="H1142" s="3" t="inlineStr">
+        <is>
+          <t>شكون كيبان emotionally unavailable ولكن كيهمو الأمر بزاف؟</t>
+        </is>
+      </c>
+      <c r="I1142" s="3" t="inlineStr"/>
+      <c r="J1142" s="3" t="inlineStr"/>
+    </row>
+    <row r="1143">
+      <c r="A1143" s="2" t="inlineStr">
+        <is>
+          <t>🆓 Free (2 Editions)</t>
+        </is>
+      </c>
+      <c r="B1143" s="2" t="inlineStr">
+        <is>
+          <t>The Free 50</t>
+        </is>
+      </c>
+      <c r="C1143" s="2" t="inlineStr">
+        <is>
+          <t>خمسون سؤال</t>
+        </is>
+      </c>
+      <c r="D1143" s="2" t="inlineStr">
+        <is>
+          <t>GROUP CHAOS</t>
+        </is>
+      </c>
+      <c r="E1143" s="2" t="inlineStr">
+        <is>
+          <t>فوضى المجموعة</t>
+        </is>
+      </c>
+      <c r="F1143" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="G1143" s="3" t="inlineStr">
+        <is>
+          <t>Who would secretly write paragraphs after an argument?</t>
+        </is>
+      </c>
+      <c r="H1143" s="3" t="inlineStr">
+        <is>
+          <t>شكون يقدر يكتب paragraph كامل من بعد الخناق؟</t>
+        </is>
+      </c>
+      <c r="I1143" s="3" t="inlineStr"/>
+      <c r="J1143" s="3" t="inlineStr"/>
+    </row>
+    <row r="1144">
+      <c r="A1144" s="2" t="inlineStr">
+        <is>
+          <t>🆓 Free (2 Editions)</t>
+        </is>
+      </c>
+      <c r="B1144" s="2" t="inlineStr">
+        <is>
+          <t>The Free 50</t>
+        </is>
+      </c>
+      <c r="C1144" s="2" t="inlineStr">
+        <is>
+          <t>خمسون سؤال</t>
+        </is>
+      </c>
+      <c r="D1144" s="2" t="inlineStr">
+        <is>
+          <t>GROUP CHAOS</t>
+        </is>
+      </c>
+      <c r="E1144" s="2" t="inlineStr">
+        <is>
+          <t>فوضى المجموعة</t>
+        </is>
+      </c>
+      <c r="F1144" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="G1144" s="3" t="inlineStr">
+        <is>
+          <t>Who seems calm but has the loudest mind?</t>
+        </is>
+      </c>
+      <c r="H1144" s="3" t="inlineStr">
+        <is>
+          <t>شكون باين هادئ ولكن عقلو loud بزاف؟</t>
+        </is>
+      </c>
+      <c r="I1144" s="3" t="inlineStr"/>
+      <c r="J1144" s="3" t="inlineStr"/>
+    </row>
+    <row r="1145">
+      <c r="A1145" s="2" t="inlineStr">
+        <is>
+          <t>🆓 Free (2 Editions)</t>
+        </is>
+      </c>
+      <c r="B1145" s="2" t="inlineStr">
+        <is>
+          <t>The Free 50</t>
+        </is>
+      </c>
+      <c r="C1145" s="2" t="inlineStr">
+        <is>
+          <t>خمسون سؤال</t>
+        </is>
+      </c>
+      <c r="D1145" s="2" t="inlineStr">
+        <is>
+          <t>THE FINAL CARDS</t>
+        </is>
+      </c>
+      <c r="E1145" s="2" t="inlineStr">
+        <is>
+          <t>البطاقات الأخيرة</t>
+        </is>
+      </c>
+      <c r="F1145" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1145" s="3" t="inlineStr">
+        <is>
+          <t>What's one thing you wish someone understood about you?</t>
+        </is>
+      </c>
+      <c r="H1145" s="3" t="inlineStr">
+        <is>
+          <t>شنو الحاجة اللي بغيتي شي حد يفهمها عليك؟</t>
+        </is>
+      </c>
+      <c r="I1145" s="3" t="inlineStr"/>
+      <c r="J1145" s="3" t="inlineStr"/>
+    </row>
+    <row r="1146">
+      <c r="A1146" s="2" t="inlineStr">
+        <is>
+          <t>🆓 Free (2 Editions)</t>
+        </is>
+      </c>
+      <c r="B1146" s="2" t="inlineStr">
+        <is>
+          <t>The Free 50</t>
+        </is>
+      </c>
+      <c r="C1146" s="2" t="inlineStr">
+        <is>
+          <t>خمسون سؤال</t>
+        </is>
+      </c>
+      <c r="D1146" s="2" t="inlineStr">
+        <is>
+          <t>THE FINAL CARDS</t>
+        </is>
+      </c>
+      <c r="E1146" s="2" t="inlineStr">
+        <is>
+          <t>البطاقات الأخيرة</t>
+        </is>
+      </c>
+      <c r="F1146" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1146" s="3" t="inlineStr">
+        <is>
+          <t>What emotion are you hiding lately?</t>
+        </is>
+      </c>
+      <c r="H1146" s="3" t="inlineStr">
+        <is>
+          <t>شنو الإحساس اللي كاتخبيه هاد الأيام؟</t>
+        </is>
+      </c>
+      <c r="I1146" s="3" t="inlineStr">
+        <is>
+          <t>Hold eye contact with someone for 10 seconds before answering.</t>
+        </is>
+      </c>
+      <c r="J1146" s="3" t="inlineStr">
+        <is>
+          <t>شوف فعيون شي واحد 10 ثواني قبل الجواب.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1147">
+      <c r="A1147" s="2" t="inlineStr">
+        <is>
+          <t>🆓 Free (2 Editions)</t>
+        </is>
+      </c>
+      <c r="B1147" s="2" t="inlineStr">
+        <is>
+          <t>The Free 50</t>
+        </is>
+      </c>
+      <c r="C1147" s="2" t="inlineStr">
+        <is>
+          <t>خمسون سؤال</t>
+        </is>
+      </c>
+      <c r="D1147" s="2" t="inlineStr">
+        <is>
+          <t>THE FINAL CARDS</t>
+        </is>
+      </c>
+      <c r="E1147" s="2" t="inlineStr">
+        <is>
+          <t>البطاقات الأخيرة</t>
+        </is>
+      </c>
+      <c r="F1147" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G1147" s="3" t="inlineStr">
+        <is>
+          <t>What kind of love do you think changes a person forever?</t>
+        </is>
+      </c>
+      <c r="H1147" s="3" t="inlineStr">
+        <is>
+          <t>شنو نوع الحب اللي كيبدل الإنسان للأبد؟</t>
+        </is>
+      </c>
+      <c r="I1147" s="3" t="inlineStr"/>
+      <c r="J1147" s="3" t="inlineStr"/>
+    </row>
+    <row r="1148">
+      <c r="A1148" s="2" t="inlineStr">
+        <is>
+          <t>🆓 Free (2 Editions)</t>
+        </is>
+      </c>
+      <c r="B1148" s="2" t="inlineStr">
+        <is>
+          <t>The Free 50</t>
+        </is>
+      </c>
+      <c r="C1148" s="2" t="inlineStr">
+        <is>
+          <t>خمسون سؤال</t>
+        </is>
+      </c>
+      <c r="D1148" s="2" t="inlineStr">
+        <is>
+          <t>THE FINAL CARDS</t>
+        </is>
+      </c>
+      <c r="E1148" s="2" t="inlineStr">
+        <is>
+          <t>البطاقات الأخيرة</t>
+        </is>
+      </c>
+      <c r="F1148" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="G1148" s="3" t="inlineStr">
+        <is>
+          <t>What truth are you avoiding these days?</t>
+        </is>
+      </c>
+      <c r="H1148" s="3" t="inlineStr">
+        <is>
+          <t>شنو الحقيقة اللي كتهرب منها دابا؟</t>
+        </is>
+      </c>
+      <c r="I1148" s="3" t="inlineStr"/>
+      <c r="J1148" s="3" t="inlineStr"/>
+    </row>
+    <row r="1149">
+      <c r="A1149" s="2" t="inlineStr">
+        <is>
+          <t>🆓 Free (2 Editions)</t>
+        </is>
+      </c>
+      <c r="B1149" s="2" t="inlineStr">
+        <is>
+          <t>The Free 50</t>
+        </is>
+      </c>
+      <c r="C1149" s="2" t="inlineStr">
+        <is>
+          <t>خمسون سؤال</t>
+        </is>
+      </c>
+      <c r="D1149" s="2" t="inlineStr">
+        <is>
+          <t>THE FINAL CARDS</t>
+        </is>
+      </c>
+      <c r="E1149" s="2" t="inlineStr">
+        <is>
+          <t>البطاقات الأخيرة</t>
+        </is>
+      </c>
+      <c r="F1149" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G1149" s="3" t="inlineStr">
+        <is>
+          <t>What's something you need emotionally right now?</t>
+        </is>
+      </c>
+      <c r="H1149" s="3" t="inlineStr">
+        <is>
+          <t>شنو الحاجة اللي محتاجها نفسياً دابا؟</t>
+        </is>
+      </c>
+      <c r="I1149" s="3" t="inlineStr"/>
+      <c r="J1149" s="3" t="inlineStr"/>
+    </row>
+    <row r="1150">
+      <c r="A1150" s="2" t="inlineStr">
+        <is>
+          <t>🆓 Free (2 Editions)</t>
+        </is>
+      </c>
+      <c r="B1150" s="2" t="inlineStr">
+        <is>
+          <t>The Free 50</t>
+        </is>
+      </c>
+      <c r="C1150" s="2" t="inlineStr">
+        <is>
+          <t>خمسون سؤال</t>
+        </is>
+      </c>
+      <c r="D1150" s="2" t="inlineStr">
+        <is>
+          <t>THE FINAL CARDS</t>
+        </is>
+      </c>
+      <c r="E1150" s="2" t="inlineStr">
+        <is>
+          <t>البطاقات الأخيرة</t>
+        </is>
+      </c>
+      <c r="F1150" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="G1150" s="3" t="inlineStr">
+        <is>
+          <t>What version of yourself are you trying to become?</t>
+        </is>
+      </c>
+      <c r="H1150" s="3" t="inlineStr">
+        <is>
+          <t>شنو النسخة منك اللي كتحاول توليها؟</t>
+        </is>
+      </c>
+      <c r="I1150" s="3" t="inlineStr">
+        <is>
+          <t>Describe your current life in 3 emotional words.</t>
+        </is>
+      </c>
+      <c r="J1150" s="3" t="inlineStr">
+        <is>
+          <t>وصف حياتك دابا بـ3 كلمات عاطفية.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1151">
+      <c r="A1151" s="2" t="inlineStr">
+        <is>
+          <t>🆓 Free (2 Editions)</t>
+        </is>
+      </c>
+      <c r="B1151" s="2" t="inlineStr">
+        <is>
+          <t>The Free 50</t>
+        </is>
+      </c>
+      <c r="C1151" s="2" t="inlineStr">
+        <is>
+          <t>خمسون سؤال</t>
+        </is>
+      </c>
+      <c r="D1151" s="2" t="inlineStr">
+        <is>
+          <t>THE FINAL CARDS</t>
+        </is>
+      </c>
+      <c r="E1151" s="2" t="inlineStr">
+        <is>
+          <t>البطاقات الأخيرة</t>
+        </is>
+      </c>
+      <c r="F1151" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="G1151" s="3" t="inlineStr">
+        <is>
+          <t>What scares you most about the future?</t>
+        </is>
+      </c>
+      <c r="H1151" s="3" t="inlineStr">
+        <is>
+          <t>شنو أكثر حاجة كتخوفك فالمستقبل؟</t>
+        </is>
+      </c>
+      <c r="I1151" s="3" t="inlineStr"/>
+      <c r="J1151" s="3" t="inlineStr"/>
+    </row>
+    <row r="1152">
+      <c r="A1152" s="2" t="inlineStr">
+        <is>
+          <t>🆓 Free (2 Editions)</t>
+        </is>
+      </c>
+      <c r="B1152" s="2" t="inlineStr">
+        <is>
+          <t>The Free 50</t>
+        </is>
+      </c>
+      <c r="C1152" s="2" t="inlineStr">
+        <is>
+          <t>خمسون سؤال</t>
+        </is>
+      </c>
+      <c r="D1152" s="2" t="inlineStr">
+        <is>
+          <t>THE FINAL CARDS</t>
+        </is>
+      </c>
+      <c r="E1152" s="2" t="inlineStr">
+        <is>
+          <t>البطاقات الأخيرة</t>
+        </is>
+      </c>
+      <c r="F1152" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="G1152" s="3" t="inlineStr">
+        <is>
+          <t>What memory changed you emotionally forever?</t>
+        </is>
+      </c>
+      <c r="H1152" s="3" t="inlineStr">
+        <is>
+          <t>شنو الذكرى اللي بدلاتك نفسياً للأبد؟</t>
+        </is>
+      </c>
+      <c r="I1152" s="3" t="inlineStr"/>
+      <c r="J1152" s="3" t="inlineStr"/>
+    </row>
+    <row r="1153">
+      <c r="A1153" s="2" t="inlineStr">
+        <is>
+          <t>🆓 Free (2 Editions)</t>
+        </is>
+      </c>
+      <c r="B1153" s="2" t="inlineStr">
+        <is>
+          <t>The Free 50</t>
+        </is>
+      </c>
+      <c r="C1153" s="2" t="inlineStr">
+        <is>
+          <t>خمسون سؤال</t>
+        </is>
+      </c>
+      <c r="D1153" s="2" t="inlineStr">
+        <is>
+          <t>THE FINAL CARDS</t>
+        </is>
+      </c>
+      <c r="E1153" s="2" t="inlineStr">
+        <is>
+          <t>البطاقات الأخيرة</t>
+        </is>
+      </c>
+      <c r="F1153" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="G1153" s="3" t="inlineStr">
+        <is>
+          <t>What do you think people feel when they meet you?</t>
+        </is>
+      </c>
+      <c r="H1153" s="3" t="inlineStr">
+        <is>
+          <t>شنو كتحس الناس كيشعرو ملي كيلقاوك؟</t>
+        </is>
+      </c>
+      <c r="I1153" s="3" t="inlineStr"/>
+      <c r="J1153" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
@@ -61767,14 +63764,14 @@
         </is>
       </c>
       <c r="C2" s="14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>140</v>
+        <v>186</v>
       </c>
       <c r="E2" s="15" t="inlineStr">
         <is>
-          <t>Talking Stage, Friends</t>
+          <t>Talking Stage, Friends, The Free 50</t>
         </is>
       </c>
     </row>
@@ -61882,14 +63879,14 @@
         </is>
       </c>
       <c r="C7" s="24" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D7" s="24" t="n">
-        <v>1106</v>
+        <v>1152</v>
       </c>
       <c r="E7" s="25" t="inlineStr">
         <is>
-          <t>Talking Stage, Couples, Married, Friends, 18+ Unfiltered, Still Us, Engaged, Secret Files, Family, Between Us, Overthinkers, Healing, Solo Edition, Masks, Love Yourself, Future, Red &amp; Green Flags, Girls Night, Who Knows Me Best?, First Impression, Artist Edition</t>
+          <t>Talking Stage, Couples, Married, Friends, 18+ Unfiltered, Still Us, Engaged, Secret Files, Family, Between Us, Overthinkers, Healing, Solo Edition, Masks, Love Yourself, Future, Red &amp; Green Flags, Girls Night, Who Knows Me Best?, First Impression, Artist Edition, The Free 50</t>
         </is>
       </c>
     </row>
@@ -68408,13 +70405,1379 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G47"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="5" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Category (EN)</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Category (AR)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Question (English)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Question (Arabic)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Challenge (EN)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Challenge (AR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="38" t="inlineStr">
+        <is>
+          <t>FUN &amp; CHAOS</t>
+        </is>
+      </c>
+      <c r="B2" s="38" t="inlineStr">
+        <is>
+          <t>الضحك والفوضى</t>
+        </is>
+      </c>
+      <c r="C2" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="38" t="inlineStr">
+        <is>
+          <t>What's your most delusional dream life?</t>
+        </is>
+      </c>
+      <c r="E2" s="38" t="inlineStr">
+        <is>
+          <t>شنو الحياة delulu اللي كتحلم بها؟</t>
+        </is>
+      </c>
+      <c r="F2" s="38" t="inlineStr"/>
+      <c r="G2" s="38" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="38" t="inlineStr">
+        <is>
+          <t>FUN &amp; CHAOS</t>
+        </is>
+      </c>
+      <c r="B3" s="38" t="inlineStr">
+        <is>
+          <t>الضحك والفوضى</t>
+        </is>
+      </c>
+      <c r="C3" s="39" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" s="38" t="inlineStr">
+        <is>
+          <t>Who here looks innocent but probably isn't?</t>
+        </is>
+      </c>
+      <c r="E3" s="38" t="inlineStr">
+        <is>
+          <t>شكون هنا باين innocent ولكن غالباً لا؟</t>
+        </is>
+      </c>
+      <c r="F3" s="38" t="inlineStr"/>
+      <c r="G3" s="38" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="38" t="inlineStr">
+        <is>
+          <t>FUN &amp; CHAOS</t>
+        </is>
+      </c>
+      <c r="B4" s="38" t="inlineStr">
+        <is>
+          <t>الضحك والفوضى</t>
+        </is>
+      </c>
+      <c r="C4" s="39" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" s="38" t="inlineStr">
+        <is>
+          <t>What's the weirdest thing you did because of emotions?</t>
+        </is>
+      </c>
+      <c r="E4" s="38" t="inlineStr">
+        <is>
+          <t>شنو أغرب حاجة درتيها بسبب المشاعر؟</t>
+        </is>
+      </c>
+      <c r="F4" s="38" t="inlineStr">
+        <is>
+          <t>Act your most dramatic emotional moment.</t>
+        </is>
+      </c>
+      <c r="G4" s="38" t="inlineStr">
+        <is>
+          <t>مثل أكثر لحظة درامية عشتها.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="38" t="inlineStr">
+        <is>
+          <t>FUN &amp; CHAOS</t>
+        </is>
+      </c>
+      <c r="B5" s="38" t="inlineStr">
+        <is>
+          <t>الضحك والفوضى</t>
+        </is>
+      </c>
+      <c r="C5" s="39" t="n">
+        <v>4</v>
+      </c>
+      <c r="D5" s="38" t="inlineStr">
+        <is>
+          <t>What's your biggest \</t>
+        </is>
+      </c>
+      <c r="E5" s="38" t="inlineStr">
+        <is>
+          <t>شنو أكبر عادة كتبيّن أنك محتاج attention؟</t>
+        </is>
+      </c>
+      <c r="F5" s="38" t="inlineStr"/>
+      <c r="G5" s="38" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="38" t="inlineStr">
+        <is>
+          <t>FUN &amp; CHAOS</t>
+        </is>
+      </c>
+      <c r="B6" s="38" t="inlineStr">
+        <is>
+          <t>الضحك والفوضى</t>
+        </is>
+      </c>
+      <c r="C6" s="39" t="n">
+        <v>5</v>
+      </c>
+      <c r="D6" s="38" t="inlineStr">
+        <is>
+          <t>Who would survive a horror movie here?</t>
+        </is>
+      </c>
+      <c r="E6" s="38" t="inlineStr">
+        <is>
+          <t>شكون يقدر ينجا ففيلم رعب هنا؟</t>
+        </is>
+      </c>
+      <c r="F6" s="38" t="inlineStr"/>
+      <c r="G6" s="38" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="38" t="inlineStr">
+        <is>
+          <t>FUN &amp; CHAOS</t>
+        </is>
+      </c>
+      <c r="B7" s="38" t="inlineStr">
+        <is>
+          <t>الضحك والفوضى</t>
+        </is>
+      </c>
+      <c r="C7" s="39" t="n">
+        <v>6</v>
+      </c>
+      <c r="D7" s="38" t="inlineStr">
+        <is>
+          <t>What's something embarrassing you still think about at 3AM?</t>
+        </is>
+      </c>
+      <c r="E7" s="38" t="inlineStr">
+        <is>
+          <t>شنو الحاجة المحرجة اللي باقي كتفكر فيها فالليل؟</t>
+        </is>
+      </c>
+      <c r="F7" s="38" t="inlineStr"/>
+      <c r="G7" s="38" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="38" t="inlineStr">
+        <is>
+          <t>FUN &amp; CHAOS</t>
+        </is>
+      </c>
+      <c r="B8" s="38" t="inlineStr">
+        <is>
+          <t>الضحك والفوضى</t>
+        </is>
+      </c>
+      <c r="C8" s="39" t="n">
+        <v>7</v>
+      </c>
+      <c r="D8" s="38" t="inlineStr">
+        <is>
+          <t>What energy do you bring into a room?</t>
+        </is>
+      </c>
+      <c r="E8" s="38" t="inlineStr">
+        <is>
+          <t>شنو الطاقة اللي كتجيب لأي بلاصة؟</t>
+        </is>
+      </c>
+      <c r="F8" s="38" t="inlineStr">
+        <is>
+          <t>Everyone describes you in one chaotic word.</t>
+        </is>
+      </c>
+      <c r="G8" s="38" t="inlineStr">
+        <is>
+          <t>كل واحد يوصفك بكلمة chaotic وحدة.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="38" t="inlineStr">
+        <is>
+          <t>FUN &amp; CHAOS</t>
+        </is>
+      </c>
+      <c r="B9" s="38" t="inlineStr">
+        <is>
+          <t>الضحك والفوضى</t>
+        </is>
+      </c>
+      <c r="C9" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="D9" s="38" t="inlineStr">
+        <is>
+          <t>What's your funniest toxic trait?</t>
+        </is>
+      </c>
+      <c r="E9" s="38" t="inlineStr">
+        <is>
+          <t>شنو أضحك toxic trait عندك؟</t>
+        </is>
+      </c>
+      <c r="F9" s="38" t="inlineStr"/>
+      <c r="G9" s="38" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="38" t="inlineStr">
+        <is>
+          <t>FUN &amp; CHAOS</t>
+        </is>
+      </c>
+      <c r="B10" s="38" t="inlineStr">
+        <is>
+          <t>الضحك والفوضى</t>
+        </is>
+      </c>
+      <c r="C10" s="39" t="n">
+        <v>9</v>
+      </c>
+      <c r="D10" s="38" t="inlineStr">
+        <is>
+          <t>What's your \</t>
+        </is>
+      </c>
+      <c r="E10" s="38" t="inlineStr">
+        <is>
+          <t>شنو الأغنية اللي كتحسسك main character؟</t>
+        </is>
+      </c>
+      <c r="F10" s="38" t="inlineStr"/>
+      <c r="G10" s="38" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="38" t="inlineStr">
+        <is>
+          <t>FUN &amp; CHAOS</t>
+        </is>
+      </c>
+      <c r="B11" s="38" t="inlineStr">
+        <is>
+          <t>الضحك والفوضى</t>
+        </is>
+      </c>
+      <c r="C11" s="39" t="n">
+        <v>10</v>
+      </c>
+      <c r="D11" s="38" t="inlineStr">
+        <is>
+          <t>What's the dumbest reason you cried for?</t>
+        </is>
+      </c>
+      <c r="E11" s="38" t="inlineStr">
+        <is>
+          <t>شنو أغبى سبب بكيت عليه؟</t>
+        </is>
+      </c>
+      <c r="F11" s="38" t="inlineStr"/>
+      <c r="G11" s="38" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="38" t="inlineStr">
+        <is>
+          <t>LOVE &amp; ATTRACTION</t>
+        </is>
+      </c>
+      <c r="B12" s="38" t="inlineStr">
+        <is>
+          <t>الحب والجذب</t>
+        </is>
+      </c>
+      <c r="C12" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="38" t="inlineStr">
+        <is>
+          <t>What kind of love secretly scares you?</t>
+        </is>
+      </c>
+      <c r="E12" s="38" t="inlineStr">
+        <is>
+          <t>شنو نوع الحب اللي كيخوفك فالسر؟</t>
+        </is>
+      </c>
+      <c r="F12" s="38" t="inlineStr"/>
+      <c r="G12" s="38" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="38" t="inlineStr">
+        <is>
+          <t>LOVE &amp; ATTRACTION</t>
+        </is>
+      </c>
+      <c r="B13" s="38" t="inlineStr">
+        <is>
+          <t>الحب والجذب</t>
+        </is>
+      </c>
+      <c r="C13" s="39" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" s="38" t="inlineStr">
+        <is>
+          <t>What instantly gives you butterflies?</t>
+        </is>
+      </c>
+      <c r="E13" s="38" t="inlineStr">
+        <is>
+          <t>شنو الحاجة اللي كتجيب ليك butterflies فوراً؟</t>
+        </is>
+      </c>
+      <c r="F13" s="38" t="inlineStr">
+        <is>
+          <t>Describe your ideal love like a movie scene.</t>
+        </is>
+      </c>
+      <c r="G13" s="38" t="inlineStr">
+        <is>
+          <t>وصف الحب المثالي بحال مشهد فيلم.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="38" t="inlineStr">
+        <is>
+          <t>LOVE &amp; ATTRACTION</t>
+        </is>
+      </c>
+      <c r="B14" s="38" t="inlineStr">
+        <is>
+          <t>الحب والجذب</t>
+        </is>
+      </c>
+      <c r="C14" s="39" t="n">
+        <v>3</v>
+      </c>
+      <c r="D14" s="38" t="inlineStr">
+        <is>
+          <t>Would you rather be adored peacefully or loved obsessively?</t>
+        </is>
+      </c>
+      <c r="E14" s="38" t="inlineStr">
+        <is>
+          <t>تفضل يتحبّوك بهدوء ولا بجنون؟</t>
+        </is>
+      </c>
+      <c r="F14" s="38" t="inlineStr"/>
+      <c r="G14" s="38" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="38" t="inlineStr">
+        <is>
+          <t>LOVE &amp; ATTRACTION</t>
+        </is>
+      </c>
+      <c r="B15" s="38" t="inlineStr">
+        <is>
+          <t>الحب والجذب</t>
+        </is>
+      </c>
+      <c r="C15" s="39" t="n">
+        <v>4</v>
+      </c>
+      <c r="D15" s="38" t="inlineStr">
+        <is>
+          <t>What's your toxic romantic habit?</t>
+        </is>
+      </c>
+      <c r="E15" s="38" t="inlineStr">
+        <is>
+          <t>شنو العادة السامة ديالك فالحب؟</t>
+        </is>
+      </c>
+      <c r="F15" s="38" t="inlineStr"/>
+      <c r="G15" s="38" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="38" t="inlineStr">
+        <is>
+          <t>LOVE &amp; ATTRACTION</t>
+        </is>
+      </c>
+      <c r="B16" s="38" t="inlineStr">
+        <is>
+          <t>الحب والجذب</t>
+        </is>
+      </c>
+      <c r="C16" s="39" t="n">
+        <v>5</v>
+      </c>
+      <c r="D16" s="38" t="inlineStr">
+        <is>
+          <t>What kind of text can ruin your mood instantly?</t>
+        </is>
+      </c>
+      <c r="E16" s="38" t="inlineStr">
+        <is>
+          <t>شنو نوع المساج اللي يقدر يخسر ليك المود فوراً؟</t>
+        </is>
+      </c>
+      <c r="F16" s="38" t="inlineStr"/>
+      <c r="G16" s="38" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="38" t="inlineStr">
+        <is>
+          <t>LOVE &amp; ATTRACTION</t>
+        </is>
+      </c>
+      <c r="B17" s="38" t="inlineStr">
+        <is>
+          <t>الحب والجذب</t>
+        </is>
+      </c>
+      <c r="C17" s="39" t="n">
+        <v>6</v>
+      </c>
+      <c r="D17" s="38" t="inlineStr">
+        <is>
+          <t>What's something romantic you pretend not to want?</t>
+        </is>
+      </c>
+      <c r="E17" s="38" t="inlineStr">
+        <is>
+          <t>شنو الحاجة الرومانسية اللي كتدير راسك ما باغيهاش؟</t>
+        </is>
+      </c>
+      <c r="F17" s="38" t="inlineStr"/>
+      <c r="G17" s="38" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="38" t="inlineStr">
+        <is>
+          <t>LOVE &amp; ATTRACTION</t>
+        </is>
+      </c>
+      <c r="B18" s="38" t="inlineStr">
+        <is>
+          <t>الحب والجذب</t>
+        </is>
+      </c>
+      <c r="C18" s="39" t="n">
+        <v>7</v>
+      </c>
+      <c r="D18" s="38" t="inlineStr">
+        <is>
+          <t>What's your biggest fear in relationships?</t>
+        </is>
+      </c>
+      <c r="E18" s="38" t="inlineStr">
+        <is>
+          <t>شنو أكبر خوف عندك فالعلاقات؟</t>
+        </is>
+      </c>
+      <c r="F18" s="38" t="inlineStr"/>
+      <c r="G18" s="38" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="38" t="inlineStr">
+        <is>
+          <t>LOVE &amp; ATTRACTION</t>
+        </is>
+      </c>
+      <c r="B19" s="38" t="inlineStr">
+        <is>
+          <t>الحب والجذب</t>
+        </is>
+      </c>
+      <c r="C19" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="D19" s="38" t="inlineStr">
+        <is>
+          <t>What makes someone emotionally attractive to you?</t>
+        </is>
+      </c>
+      <c r="E19" s="38" t="inlineStr">
+        <is>
+          <t>شنو كيخلي الشخص جذاب نفسياً؟</t>
+        </is>
+      </c>
+      <c r="F19" s="38" t="inlineStr"/>
+      <c r="G19" s="38" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="38" t="inlineStr">
+        <is>
+          <t>LOVE &amp; ATTRACTION</t>
+        </is>
+      </c>
+      <c r="B20" s="38" t="inlineStr">
+        <is>
+          <t>الحب والجذب</t>
+        </is>
+      </c>
+      <c r="C20" s="39" t="n">
+        <v>9</v>
+      </c>
+      <c r="D20" s="38" t="inlineStr">
+        <is>
+          <t>What kind of love story fits your soul?</t>
+        </is>
+      </c>
+      <c r="E20" s="38" t="inlineStr">
+        <is>
+          <t>شنو قصة الحب اللي كتشبه روحك؟</t>
+        </is>
+      </c>
+      <c r="F20" s="38" t="inlineStr"/>
+      <c r="G20" s="38" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="38" t="inlineStr">
+        <is>
+          <t>DEEP THOUGHTS</t>
+        </is>
+      </c>
+      <c r="B21" s="38" t="inlineStr">
+        <is>
+          <t>أعماق التفكير</t>
+        </is>
+      </c>
+      <c r="C21" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="38" t="inlineStr">
+        <is>
+          <t>What thought ruins your peace the most?</t>
+        </is>
+      </c>
+      <c r="E21" s="38" t="inlineStr">
+        <is>
+          <t>شنو الفكرة اللي كتخرب عليك الراحة أكثر؟</t>
+        </is>
+      </c>
+      <c r="F21" s="38" t="inlineStr"/>
+      <c r="G21" s="38" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="38" t="inlineStr">
+        <is>
+          <t>DEEP THOUGHTS</t>
+        </is>
+      </c>
+      <c r="B22" s="38" t="inlineStr">
+        <is>
+          <t>أعماق التفكير</t>
+        </is>
+      </c>
+      <c r="C22" s="39" t="n">
+        <v>2</v>
+      </c>
+      <c r="D22" s="38" t="inlineStr">
+        <is>
+          <t>What do you hide behind your personality?</t>
+        </is>
+      </c>
+      <c r="E22" s="38" t="inlineStr">
+        <is>
+          <t>شنو كتخبي ورا شخصيتك؟</t>
+        </is>
+      </c>
+      <c r="F22" s="38" t="inlineStr"/>
+      <c r="G22" s="38" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="38" t="inlineStr">
+        <is>
+          <t>DEEP THOUGHTS</t>
+        </is>
+      </c>
+      <c r="B23" s="38" t="inlineStr">
+        <is>
+          <t>أعماق التفكير</t>
+        </is>
+      </c>
+      <c r="C23" s="39" t="n">
+        <v>3</v>
+      </c>
+      <c r="D23" s="38" t="inlineStr">
+        <is>
+          <t>What version of yourself are you grieving?</t>
+        </is>
+      </c>
+      <c r="E23" s="38" t="inlineStr">
+        <is>
+          <t>شنو النسخة منك اللي كتحزن عليها؟</t>
+        </is>
+      </c>
+      <c r="F23" s="38" t="inlineStr"/>
+      <c r="G23" s="38" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="38" t="inlineStr">
+        <is>
+          <t>DEEP THOUGHTS</t>
+        </is>
+      </c>
+      <c r="B24" s="38" t="inlineStr">
+        <is>
+          <t>أعماق التفكير</t>
+        </is>
+      </c>
+      <c r="C24" s="39" t="n">
+        <v>4</v>
+      </c>
+      <c r="D24" s="38" t="inlineStr">
+        <is>
+          <t>What emotional wound still affects you quietly?</t>
+        </is>
+      </c>
+      <c r="E24" s="38" t="inlineStr">
+        <is>
+          <t>شنو الجرح اللي باقي كيأثر عليك بصمت؟</t>
+        </is>
+      </c>
+      <c r="F24" s="38" t="inlineStr"/>
+      <c r="G24" s="38" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="38" t="inlineStr">
+        <is>
+          <t>DEEP THOUGHTS</t>
+        </is>
+      </c>
+      <c r="B25" s="38" t="inlineStr">
+        <is>
+          <t>أعماق التفكير</t>
+        </is>
+      </c>
+      <c r="C25" s="39" t="n">
+        <v>5</v>
+      </c>
+      <c r="D25" s="38" t="inlineStr">
+        <is>
+          <t>What do you wish people understood about you?</t>
+        </is>
+      </c>
+      <c r="E25" s="38" t="inlineStr">
+        <is>
+          <t>شنو بغيتي الناس يفهموه عليك؟</t>
+        </is>
+      </c>
+      <c r="F25" s="38" t="inlineStr"/>
+      <c r="G25" s="38" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="38" t="inlineStr">
+        <is>
+          <t>DEEP THOUGHTS</t>
+        </is>
+      </c>
+      <c r="B26" s="38" t="inlineStr">
+        <is>
+          <t>أعماق التفكير</t>
+        </is>
+      </c>
+      <c r="C26" s="39" t="n">
+        <v>6</v>
+      </c>
+      <c r="D26" s="38" t="inlineStr">
+        <is>
+          <t>What's a fear you never say out loud?</t>
+        </is>
+      </c>
+      <c r="E26" s="38" t="inlineStr">
+        <is>
+          <t>شنو الخوف اللي ما كتقولوش بصوت عالي؟</t>
+        </is>
+      </c>
+      <c r="F26" s="38" t="inlineStr">
+        <is>
+          <t>Silence round — answer with no jokes allowed.</t>
+        </is>
+      </c>
+      <c r="G26" s="38" t="inlineStr">
+        <is>
+          <t>جولة الصمت — جاوب بلا ضحك ولا هزار.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="38" t="inlineStr">
+        <is>
+          <t>DEEP THOUGHTS</t>
+        </is>
+      </c>
+      <c r="B27" s="38" t="inlineStr">
+        <is>
+          <t>أعماق التفكير</t>
+        </is>
+      </c>
+      <c r="C27" s="39" t="n">
+        <v>7</v>
+      </c>
+      <c r="D27" s="38" t="inlineStr">
+        <is>
+          <t>What kind of loneliness do you experience?</t>
+        </is>
+      </c>
+      <c r="E27" s="38" t="inlineStr">
+        <is>
+          <t>شنو نوع الوحدة اللي كتحس بها؟</t>
+        </is>
+      </c>
+      <c r="F27" s="38" t="inlineStr"/>
+      <c r="G27" s="38" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="38" t="inlineStr">
+        <is>
+          <t>DEEP THOUGHTS</t>
+        </is>
+      </c>
+      <c r="B28" s="38" t="inlineStr">
+        <is>
+          <t>أعماق التفكير</t>
+        </is>
+      </c>
+      <c r="C28" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="D28" s="38" t="inlineStr">
+        <is>
+          <t>What emotion do you struggle to express?</t>
+        </is>
+      </c>
+      <c r="E28" s="38" t="inlineStr">
+        <is>
+          <t>شنو الإحساس اللي صعيب عليك تعبر عليه؟</t>
+        </is>
+      </c>
+      <c r="F28" s="38" t="inlineStr"/>
+      <c r="G28" s="38" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="38" t="inlineStr">
+        <is>
+          <t>DEEP THOUGHTS</t>
+        </is>
+      </c>
+      <c r="B29" s="38" t="inlineStr">
+        <is>
+          <t>أعماق التفكير</t>
+        </is>
+      </c>
+      <c r="C29" s="39" t="n">
+        <v>9</v>
+      </c>
+      <c r="D29" s="38" t="inlineStr">
+        <is>
+          <t>What do you overthink the most at night?</t>
+        </is>
+      </c>
+      <c r="E29" s="38" t="inlineStr">
+        <is>
+          <t>شنو كتكتر التفكير فيه فالليل؟</t>
+        </is>
+      </c>
+      <c r="F29" s="38" t="inlineStr"/>
+      <c r="G29" s="38" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="38" t="inlineStr">
+        <is>
+          <t>GROUP CHAOS</t>
+        </is>
+      </c>
+      <c r="B30" s="38" t="inlineStr">
+        <is>
+          <t>فوضى المجموعة</t>
+        </is>
+      </c>
+      <c r="C30" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="38" t="inlineStr">
+        <is>
+          <t>Who here hides their emotions the best?</t>
+        </is>
+      </c>
+      <c r="E30" s="38" t="inlineStr">
+        <is>
+          <t>شكون هنا كايخبي مشاعرو مزيان؟</t>
+        </is>
+      </c>
+      <c r="F30" s="38" t="inlineStr"/>
+      <c r="G30" s="38" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="38" t="inlineStr">
+        <is>
+          <t>GROUP CHAOS</t>
+        </is>
+      </c>
+      <c r="B31" s="38" t="inlineStr">
+        <is>
+          <t>فوضى المجموعة</t>
+        </is>
+      </c>
+      <c r="C31" s="39" t="n">
+        <v>2</v>
+      </c>
+      <c r="D31" s="38" t="inlineStr">
+        <is>
+          <t>Who would fall in love the fastest?</t>
+        </is>
+      </c>
+      <c r="E31" s="38" t="inlineStr">
+        <is>
+          <t>شكون يقدر يحب بسرعة أكثر؟</t>
+        </is>
+      </c>
+      <c r="F31" s="38" t="inlineStr">
+        <is>
+          <t>Vote anonymously.</t>
+        </is>
+      </c>
+      <c r="G31" s="38" t="inlineStr">
+        <is>
+          <t>صوتو anonymously.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="38" t="inlineStr">
+        <is>
+          <t>GROUP CHAOS</t>
+        </is>
+      </c>
+      <c r="B32" s="38" t="inlineStr">
+        <is>
+          <t>فوضى المجموعة</t>
+        </is>
+      </c>
+      <c r="C32" s="39" t="n">
+        <v>3</v>
+      </c>
+      <c r="D32" s="38" t="inlineStr">
+        <is>
+          <t>Who looks soft but is emotionally dangerous?</t>
+        </is>
+      </c>
+      <c r="E32" s="38" t="inlineStr">
+        <is>
+          <t>شكون باين حنين ولكن dangerous عاطفياً؟</t>
+        </is>
+      </c>
+      <c r="F32" s="38" t="inlineStr"/>
+      <c r="G32" s="38" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="38" t="inlineStr">
+        <is>
+          <t>GROUP CHAOS</t>
+        </is>
+      </c>
+      <c r="B33" s="38" t="inlineStr">
+        <is>
+          <t>فوضى المجموعة</t>
+        </is>
+      </c>
+      <c r="C33" s="39" t="n">
+        <v>4</v>
+      </c>
+      <c r="D33" s="38" t="inlineStr">
+        <is>
+          <t>Who gives heartbreak energy?</t>
+        </is>
+      </c>
+      <c r="E33" s="38" t="inlineStr">
+        <is>
+          <t>شكون كييعطي heartbreak energy؟</t>
+        </is>
+      </c>
+      <c r="F33" s="38" t="inlineStr"/>
+      <c r="G33" s="38" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="38" t="inlineStr">
+        <is>
+          <t>GROUP CHAOS</t>
+        </is>
+      </c>
+      <c r="B34" s="38" t="inlineStr">
+        <is>
+          <t>فوضى المجموعة</t>
+        </is>
+      </c>
+      <c r="C34" s="39" t="n">
+        <v>5</v>
+      </c>
+      <c r="D34" s="38" t="inlineStr">
+        <is>
+          <t>Who overthinks every text message?</t>
+        </is>
+      </c>
+      <c r="E34" s="38" t="inlineStr">
+        <is>
+          <t>شكون كيحلل كل مساج بزاف؟</t>
+        </is>
+      </c>
+      <c r="F34" s="38" t="inlineStr"/>
+      <c r="G34" s="38" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="38" t="inlineStr">
+        <is>
+          <t>GROUP CHAOS</t>
+        </is>
+      </c>
+      <c r="B35" s="38" t="inlineStr">
+        <is>
+          <t>فوضى المجموعة</t>
+        </is>
+      </c>
+      <c r="C35" s="39" t="n">
+        <v>6</v>
+      </c>
+      <c r="D35" s="38" t="inlineStr">
+        <is>
+          <t>Who would disappear after heartbreak?</t>
+        </is>
+      </c>
+      <c r="E35" s="38" t="inlineStr">
+        <is>
+          <t>شكون يقدر يختفي من بعد heartbreak؟</t>
+        </is>
+      </c>
+      <c r="F35" s="38" t="inlineStr">
+        <is>
+          <t>Everyone imitates the person they choose.</t>
+        </is>
+      </c>
+      <c r="G35" s="38" t="inlineStr">
+        <is>
+          <t>كل واحد يقلد الشخص اللي اختار.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="38" t="inlineStr">
+        <is>
+          <t>GROUP CHAOS</t>
+        </is>
+      </c>
+      <c r="B36" s="38" t="inlineStr">
+        <is>
+          <t>فوضى المجموعة</t>
+        </is>
+      </c>
+      <c r="C36" s="39" t="n">
+        <v>7</v>
+      </c>
+      <c r="D36" s="38" t="inlineStr">
+        <is>
+          <t>Who acts emotionally unavailable but actually cares deeply?</t>
+        </is>
+      </c>
+      <c r="E36" s="38" t="inlineStr">
+        <is>
+          <t>شكون كيبان emotionally unavailable ولكن كيهمو الأمر بزاف؟</t>
+        </is>
+      </c>
+      <c r="F36" s="38" t="inlineStr"/>
+      <c r="G36" s="38" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="38" t="inlineStr">
+        <is>
+          <t>GROUP CHAOS</t>
+        </is>
+      </c>
+      <c r="B37" s="38" t="inlineStr">
+        <is>
+          <t>فوضى المجموعة</t>
+        </is>
+      </c>
+      <c r="C37" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="D37" s="38" t="inlineStr">
+        <is>
+          <t>Who would secretly write paragraphs after an argument?</t>
+        </is>
+      </c>
+      <c r="E37" s="38" t="inlineStr">
+        <is>
+          <t>شكون يقدر يكتب paragraph كامل من بعد الخناق؟</t>
+        </is>
+      </c>
+      <c r="F37" s="38" t="inlineStr"/>
+      <c r="G37" s="38" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="38" t="inlineStr">
+        <is>
+          <t>GROUP CHAOS</t>
+        </is>
+      </c>
+      <c r="B38" s="38" t="inlineStr">
+        <is>
+          <t>فوضى المجموعة</t>
+        </is>
+      </c>
+      <c r="C38" s="39" t="n">
+        <v>9</v>
+      </c>
+      <c r="D38" s="38" t="inlineStr">
+        <is>
+          <t>Who seems calm but has the loudest mind?</t>
+        </is>
+      </c>
+      <c r="E38" s="38" t="inlineStr">
+        <is>
+          <t>شكون باين هادئ ولكن عقلو loud بزاف؟</t>
+        </is>
+      </c>
+      <c r="F38" s="38" t="inlineStr"/>
+      <c r="G38" s="38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="38" t="inlineStr">
+        <is>
+          <t>THE FINAL CARDS</t>
+        </is>
+      </c>
+      <c r="B39" s="38" t="inlineStr">
+        <is>
+          <t>البطاقات الأخيرة</t>
+        </is>
+      </c>
+      <c r="C39" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" s="38" t="inlineStr">
+        <is>
+          <t>What's one thing you wish someone understood about you?</t>
+        </is>
+      </c>
+      <c r="E39" s="38" t="inlineStr">
+        <is>
+          <t>شنو الحاجة اللي بغيتي شي حد يفهمها عليك؟</t>
+        </is>
+      </c>
+      <c r="F39" s="38" t="inlineStr"/>
+      <c r="G39" s="38" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="38" t="inlineStr">
+        <is>
+          <t>THE FINAL CARDS</t>
+        </is>
+      </c>
+      <c r="B40" s="38" t="inlineStr">
+        <is>
+          <t>البطاقات الأخيرة</t>
+        </is>
+      </c>
+      <c r="C40" s="39" t="n">
+        <v>2</v>
+      </c>
+      <c r="D40" s="38" t="inlineStr">
+        <is>
+          <t>What emotion are you hiding lately?</t>
+        </is>
+      </c>
+      <c r="E40" s="38" t="inlineStr">
+        <is>
+          <t>شنو الإحساس اللي كاتخبيه هاد الأيام؟</t>
+        </is>
+      </c>
+      <c r="F40" s="38" t="inlineStr">
+        <is>
+          <t>Hold eye contact with someone for 10 seconds before answering.</t>
+        </is>
+      </c>
+      <c r="G40" s="38" t="inlineStr">
+        <is>
+          <t>شوف فعيون شي واحد 10 ثواني قبل الجواب.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="38" t="inlineStr">
+        <is>
+          <t>THE FINAL CARDS</t>
+        </is>
+      </c>
+      <c r="B41" s="38" t="inlineStr">
+        <is>
+          <t>البطاقات الأخيرة</t>
+        </is>
+      </c>
+      <c r="C41" s="39" t="n">
+        <v>3</v>
+      </c>
+      <c r="D41" s="38" t="inlineStr">
+        <is>
+          <t>What kind of love do you think changes a person forever?</t>
+        </is>
+      </c>
+      <c r="E41" s="38" t="inlineStr">
+        <is>
+          <t>شنو نوع الحب اللي كيبدل الإنسان للأبد؟</t>
+        </is>
+      </c>
+      <c r="F41" s="38" t="inlineStr"/>
+      <c r="G41" s="38" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="38" t="inlineStr">
+        <is>
+          <t>THE FINAL CARDS</t>
+        </is>
+      </c>
+      <c r="B42" s="38" t="inlineStr">
+        <is>
+          <t>البطاقات الأخيرة</t>
+        </is>
+      </c>
+      <c r="C42" s="39" t="n">
+        <v>4</v>
+      </c>
+      <c r="D42" s="38" t="inlineStr">
+        <is>
+          <t>What truth are you avoiding these days?</t>
+        </is>
+      </c>
+      <c r="E42" s="38" t="inlineStr">
+        <is>
+          <t>شنو الحقيقة اللي كتهرب منها دابا؟</t>
+        </is>
+      </c>
+      <c r="F42" s="38" t="inlineStr"/>
+      <c r="G42" s="38" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="38" t="inlineStr">
+        <is>
+          <t>THE FINAL CARDS</t>
+        </is>
+      </c>
+      <c r="B43" s="38" t="inlineStr">
+        <is>
+          <t>البطاقات الأخيرة</t>
+        </is>
+      </c>
+      <c r="C43" s="39" t="n">
+        <v>5</v>
+      </c>
+      <c r="D43" s="38" t="inlineStr">
+        <is>
+          <t>What's something you need emotionally right now?</t>
+        </is>
+      </c>
+      <c r="E43" s="38" t="inlineStr">
+        <is>
+          <t>شنو الحاجة اللي محتاجها نفسياً دابا؟</t>
+        </is>
+      </c>
+      <c r="F43" s="38" t="inlineStr"/>
+      <c r="G43" s="38" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="38" t="inlineStr">
+        <is>
+          <t>THE FINAL CARDS</t>
+        </is>
+      </c>
+      <c r="B44" s="38" t="inlineStr">
+        <is>
+          <t>البطاقات الأخيرة</t>
+        </is>
+      </c>
+      <c r="C44" s="39" t="n">
+        <v>6</v>
+      </c>
+      <c r="D44" s="38" t="inlineStr">
+        <is>
+          <t>What version of yourself are you trying to become?</t>
+        </is>
+      </c>
+      <c r="E44" s="38" t="inlineStr">
+        <is>
+          <t>شنو النسخة منك اللي كتحاول توليها؟</t>
+        </is>
+      </c>
+      <c r="F44" s="38" t="inlineStr">
+        <is>
+          <t>Describe your current life in 3 emotional words.</t>
+        </is>
+      </c>
+      <c r="G44" s="38" t="inlineStr">
+        <is>
+          <t>وصف حياتك دابا بـ3 كلمات عاطفية.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="38" t="inlineStr">
+        <is>
+          <t>THE FINAL CARDS</t>
+        </is>
+      </c>
+      <c r="B45" s="38" t="inlineStr">
+        <is>
+          <t>البطاقات الأخيرة</t>
+        </is>
+      </c>
+      <c r="C45" s="39" t="n">
+        <v>7</v>
+      </c>
+      <c r="D45" s="38" t="inlineStr">
+        <is>
+          <t>What scares you most about the future?</t>
+        </is>
+      </c>
+      <c r="E45" s="38" t="inlineStr">
+        <is>
+          <t>شنو أكثر حاجة كتخوفك فالمستقبل؟</t>
+        </is>
+      </c>
+      <c r="F45" s="38" t="inlineStr"/>
+      <c r="G45" s="38" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="38" t="inlineStr">
+        <is>
+          <t>THE FINAL CARDS</t>
+        </is>
+      </c>
+      <c r="B46" s="38" t="inlineStr">
+        <is>
+          <t>البطاقات الأخيرة</t>
+        </is>
+      </c>
+      <c r="C46" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="D46" s="38" t="inlineStr">
+        <is>
+          <t>What memory changed you emotionally forever?</t>
+        </is>
+      </c>
+      <c r="E46" s="38" t="inlineStr">
+        <is>
+          <t>شنو الذكرى اللي بدلاتك نفسياً للأبد؟</t>
+        </is>
+      </c>
+      <c r="F46" s="38" t="inlineStr"/>
+      <c r="G46" s="38" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="38" t="inlineStr">
+        <is>
+          <t>THE FINAL CARDS</t>
+        </is>
+      </c>
+      <c r="B47" s="38" t="inlineStr">
+        <is>
+          <t>البطاقات الأخيرة</t>
+        </is>
+      </c>
+      <c r="C47" s="39" t="n">
+        <v>9</v>
+      </c>
+      <c r="D47" s="38" t="inlineStr">
+        <is>
+          <t>What do you think people feel when they meet you?</t>
+        </is>
+      </c>
+      <c r="E47" s="38" t="inlineStr">
+        <is>
+          <t>شنو كتحس الناس كيشعرو ملي كيلقاوك؟</t>
+        </is>
+      </c>
+      <c r="F47" s="38" t="inlineStr"/>
+      <c r="G47" s="38" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -69112,6 +72475,37 @@
       </c>
       <c r="G22" s="36" t="n">
         <v>40</v>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="26" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="27" t="inlineStr">
+        <is>
+          <t>The Free 50</t>
+        </is>
+      </c>
+      <c r="C23" s="27" t="inlineStr">
+        <is>
+          <t>خمسون سؤال</t>
+        </is>
+      </c>
+      <c r="D23" s="27" t="inlineStr">
+        <is>
+          <t>🆓 Free (2 Editions)</t>
+        </is>
+      </c>
+      <c r="E23" s="26" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="F23" s="26" t="n">
+        <v>5</v>
+      </c>
+      <c r="G23" s="26" t="n">
+        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>